<commit_message>
update full exact fairness experiments
</commit_message>
<xml_diff>
--- a/v3/data/raw/five_time_windows.xlsx
+++ b/v3/data/raw/five_time_windows.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jinghongmiao/Code/mvt-code/v3/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91AB409-B6F3-314E-8E4C-7B3980CA9E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9644AC14-3F78-FD47-9506-9D32193D4924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="4" xr2:uid="{80C050B1-FB2F-EF4E-8D88-071846B14504}"/>
+    <workbookView xWindow="2120" yWindow="660" windowWidth="30240" windowHeight="18880" activeTab="6" xr2:uid="{80C050B1-FB2F-EF4E-8D88-071846B14504}"/>
   </bookViews>
   <sheets>
     <sheet name="Even" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="Skewed2" sheetId="4" r:id="rId3"/>
     <sheet name="Random1" sheetId="5" r:id="rId4"/>
     <sheet name="Random2" sheetId="2" r:id="rId5"/>
+    <sheet name="Even2" sheetId="6" r:id="rId6"/>
+    <sheet name="Even3" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="11">
   <si>
     <t>Event</t>
   </si>
@@ -94,12 +96,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -129,11 +137,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9436,4 +9446,3594 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC8E905D-8FFC-D941-96F4-D3B0810C556A}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>570</v>
+      </c>
+      <c r="C2">
+        <v>810</v>
+      </c>
+      <c r="D2" s="2">
+        <v>570</v>
+      </c>
+      <c r="E2" s="2">
+        <v>810</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>570</v>
+      </c>
+      <c r="G3" s="2">
+        <v>810</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>570</v>
+      </c>
+      <c r="K3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
+        <v>570</v>
+      </c>
+      <c r="I4" s="2">
+        <v>810</v>
+      </c>
+      <c r="J4">
+        <v>570</v>
+      </c>
+      <c r="K4">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>570</v>
+      </c>
+      <c r="E5" s="3">
+        <v>810</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>570</v>
+      </c>
+      <c r="K5" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>570</v>
+      </c>
+      <c r="C6" s="2">
+        <v>810</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>570</v>
+      </c>
+      <c r="K6">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>570</v>
+      </c>
+      <c r="C7" s="2">
+        <v>810</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>570</v>
+      </c>
+      <c r="I7" s="3">
+        <v>810</v>
+      </c>
+      <c r="J7" s="3">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>0</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0</v>
+      </c>
+      <c r="D8" s="2">
+        <v>570</v>
+      </c>
+      <c r="E8" s="2">
+        <v>810</v>
+      </c>
+      <c r="F8" s="3">
+        <v>570</v>
+      </c>
+      <c r="G8" s="3">
+        <v>810</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3">
+        <v>570</v>
+      </c>
+      <c r="C9" s="3">
+        <v>810</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>570</v>
+      </c>
+      <c r="G9" s="2">
+        <v>810</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3">
+        <v>570</v>
+      </c>
+      <c r="C10" s="3">
+        <v>810</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>570</v>
+      </c>
+      <c r="K10" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
+        <v>570</v>
+      </c>
+      <c r="I11" s="2">
+        <v>810</v>
+      </c>
+      <c r="J11" s="3">
+        <v>570</v>
+      </c>
+      <c r="K11" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>570</v>
+      </c>
+      <c r="C12" s="2">
+        <v>810</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3">
+        <v>570</v>
+      </c>
+      <c r="G12" s="3">
+        <v>810</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>570</v>
+      </c>
+      <c r="E13" s="3">
+        <v>810</v>
+      </c>
+      <c r="F13" s="2">
+        <v>570</v>
+      </c>
+      <c r="G13" s="2">
+        <v>810</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2">
+        <v>570</v>
+      </c>
+      <c r="E14" s="2">
+        <v>810</v>
+      </c>
+      <c r="F14" s="3">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3">
+        <v>570</v>
+      </c>
+      <c r="K14" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>570</v>
+      </c>
+      <c r="E15" s="3">
+        <v>810</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>570</v>
+      </c>
+      <c r="I15" s="2">
+        <v>810</v>
+      </c>
+      <c r="J15" s="3">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>570</v>
+      </c>
+      <c r="E16" s="3">
+        <v>810</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>570</v>
+      </c>
+      <c r="K16" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3">
+        <v>570</v>
+      </c>
+      <c r="C17" s="3">
+        <v>810</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2">
+        <v>570</v>
+      </c>
+      <c r="G17" s="2">
+        <v>810</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3">
+        <v>0</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3">
+        <v>0</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>570</v>
+      </c>
+      <c r="G18" s="3">
+        <v>810</v>
+      </c>
+      <c r="H18" s="2">
+        <v>570</v>
+      </c>
+      <c r="I18" s="2">
+        <v>810</v>
+      </c>
+      <c r="J18" s="3">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3">
+        <v>570</v>
+      </c>
+      <c r="G19" s="3">
+        <v>810</v>
+      </c>
+      <c r="H19" s="3">
+        <v>0</v>
+      </c>
+      <c r="I19" s="3">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2">
+        <v>570</v>
+      </c>
+      <c r="K19" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2">
+        <v>570</v>
+      </c>
+      <c r="C20" s="2">
+        <v>810</v>
+      </c>
+      <c r="D20">
+        <v>570</v>
+      </c>
+      <c r="E20">
+        <v>810</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>570</v>
+      </c>
+      <c r="C21">
+        <v>810</v>
+      </c>
+      <c r="D21" s="2">
+        <v>570</v>
+      </c>
+      <c r="E21" s="2">
+        <v>810</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2">
+        <v>570</v>
+      </c>
+      <c r="C22" s="2">
+        <v>810</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>570</v>
+      </c>
+      <c r="I22">
+        <v>810</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2">
+        <v>570</v>
+      </c>
+      <c r="E23" s="2">
+        <v>810</v>
+      </c>
+      <c r="F23">
+        <v>570</v>
+      </c>
+      <c r="G23">
+        <v>810</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2">
+        <v>570</v>
+      </c>
+      <c r="G24" s="2">
+        <v>810</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>570</v>
+      </c>
+      <c r="K24">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>570</v>
+      </c>
+      <c r="E25">
+        <v>810</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2">
+        <v>570</v>
+      </c>
+      <c r="I25" s="2">
+        <v>810</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>570</v>
+      </c>
+      <c r="G26">
+        <v>810</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2">
+        <v>570</v>
+      </c>
+      <c r="K26" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>570</v>
+      </c>
+      <c r="C27">
+        <v>810</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2">
+        <v>570</v>
+      </c>
+      <c r="G27" s="2">
+        <v>810</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2">
+        <v>570</v>
+      </c>
+      <c r="I28" s="2">
+        <v>810</v>
+      </c>
+      <c r="J28">
+        <v>570</v>
+      </c>
+      <c r="K28">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>570</v>
+      </c>
+      <c r="I29">
+        <v>810</v>
+      </c>
+      <c r="J29" s="2">
+        <v>570</v>
+      </c>
+      <c r="K29" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>570</v>
+      </c>
+      <c r="C30">
+        <v>810</v>
+      </c>
+      <c r="D30" s="2">
+        <v>570</v>
+      </c>
+      <c r="E30" s="2">
+        <v>810</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2">
+        <v>570</v>
+      </c>
+      <c r="C31" s="2">
+        <v>810</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <v>570</v>
+      </c>
+      <c r="G31">
+        <v>810</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2">
+        <v>570</v>
+      </c>
+      <c r="C32" s="2">
+        <v>810</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>570</v>
+      </c>
+      <c r="K32">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>570</v>
+      </c>
+      <c r="C33">
+        <v>810</v>
+      </c>
+      <c r="D33" s="2">
+        <v>570</v>
+      </c>
+      <c r="E33" s="2">
+        <v>810</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>570</v>
+      </c>
+      <c r="G34">
+        <v>810</v>
+      </c>
+      <c r="H34" s="2">
+        <v>570</v>
+      </c>
+      <c r="I34" s="2">
+        <v>810</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35">
+        <v>570</v>
+      </c>
+      <c r="I35">
+        <v>810</v>
+      </c>
+      <c r="J35" s="2">
+        <v>570</v>
+      </c>
+      <c r="K35" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36" s="2">
+        <v>570</v>
+      </c>
+      <c r="G36" s="2">
+        <v>810</v>
+      </c>
+      <c r="H36">
+        <v>570</v>
+      </c>
+      <c r="I36">
+        <v>810</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2">
+        <v>570</v>
+      </c>
+      <c r="C37" s="2">
+        <v>810</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>570</v>
+      </c>
+      <c r="I37">
+        <v>810</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38" s="2">
+        <v>570</v>
+      </c>
+      <c r="E38" s="2">
+        <v>810</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>570</v>
+      </c>
+      <c r="I38">
+        <v>810</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39">
+        <v>0</v>
+      </c>
+      <c r="F39" s="2">
+        <v>570</v>
+      </c>
+      <c r="G39" s="2">
+        <v>810</v>
+      </c>
+      <c r="H39">
+        <v>570</v>
+      </c>
+      <c r="I39">
+        <v>810</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>0</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>570</v>
+      </c>
+      <c r="E40">
+        <v>810</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2">
+        <v>570</v>
+      </c>
+      <c r="I40" s="2">
+        <v>810</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>0</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>0</v>
+      </c>
+      <c r="F41">
+        <v>570</v>
+      </c>
+      <c r="G41">
+        <v>810</v>
+      </c>
+      <c r="H41">
+        <v>0</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41" s="2">
+        <v>570</v>
+      </c>
+      <c r="K41" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2">
+        <v>570</v>
+      </c>
+      <c r="C42" s="2">
+        <v>810</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>570</v>
+      </c>
+      <c r="K42">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>0</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43" s="2">
+        <v>570</v>
+      </c>
+      <c r="E43" s="2">
+        <v>810</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>570</v>
+      </c>
+      <c r="I43">
+        <v>810</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>570</v>
+      </c>
+      <c r="C44">
+        <v>810</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44" s="2">
+        <v>570</v>
+      </c>
+      <c r="G44" s="2">
+        <v>810</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44">
+        <v>0</v>
+      </c>
+      <c r="K44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>0</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>570</v>
+      </c>
+      <c r="E45">
+        <v>810</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45" s="2">
+        <v>570</v>
+      </c>
+      <c r="I45" s="2">
+        <v>810</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>0</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
+        <v>570</v>
+      </c>
+      <c r="I46">
+        <v>810</v>
+      </c>
+      <c r="J46" s="2">
+        <v>570</v>
+      </c>
+      <c r="K46" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>570</v>
+      </c>
+      <c r="C47">
+        <v>810</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47" s="2">
+        <v>570</v>
+      </c>
+      <c r="G47" s="2">
+        <v>810</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <v>0</v>
+      </c>
+      <c r="J47">
+        <v>0</v>
+      </c>
+      <c r="K47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>0</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48" s="2">
+        <v>570</v>
+      </c>
+      <c r="I48" s="2">
+        <v>810</v>
+      </c>
+      <c r="J48">
+        <v>570</v>
+      </c>
+      <c r="K48">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>0</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>570</v>
+      </c>
+      <c r="E49">
+        <v>810</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49" s="2">
+        <v>570</v>
+      </c>
+      <c r="K49" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2">
+        <v>570</v>
+      </c>
+      <c r="C50" s="2">
+        <v>810</v>
+      </c>
+      <c r="D50">
+        <v>570</v>
+      </c>
+      <c r="E50">
+        <v>810</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
+        <v>0</v>
+      </c>
+      <c r="H50">
+        <v>0</v>
+      </c>
+      <c r="I50">
+        <v>0</v>
+      </c>
+      <c r="J50">
+        <v>0</v>
+      </c>
+      <c r="K50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>0</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51" s="2">
+        <v>570</v>
+      </c>
+      <c r="E51" s="2">
+        <v>810</v>
+      </c>
+      <c r="F51">
+        <v>570</v>
+      </c>
+      <c r="G51">
+        <v>810</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51">
+        <v>0</v>
+      </c>
+      <c r="J51">
+        <v>0</v>
+      </c>
+      <c r="K51">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F561FCD-E65A-AA42-B671-94071C3571EB}">
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3">
+        <v>570</v>
+      </c>
+      <c r="C2" s="3">
+        <v>810</v>
+      </c>
+      <c r="D2" s="3">
+        <v>570</v>
+      </c>
+      <c r="E2" s="3">
+        <v>810</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>570</v>
+      </c>
+      <c r="K2" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3">
+        <v>570</v>
+      </c>
+      <c r="G3" s="3">
+        <v>810</v>
+      </c>
+      <c r="H3" s="2">
+        <v>570</v>
+      </c>
+      <c r="I3" s="2">
+        <v>810</v>
+      </c>
+      <c r="J3" s="3">
+        <v>570</v>
+      </c>
+      <c r="K3" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>570</v>
+      </c>
+      <c r="G4" s="2">
+        <v>810</v>
+      </c>
+      <c r="H4" s="3">
+        <v>570</v>
+      </c>
+      <c r="I4" s="3">
+        <v>810</v>
+      </c>
+      <c r="J4" s="3">
+        <v>570</v>
+      </c>
+      <c r="K4" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>570</v>
+      </c>
+      <c r="C5" s="2">
+        <v>810</v>
+      </c>
+      <c r="D5" s="3">
+        <v>570</v>
+      </c>
+      <c r="E5" s="3">
+        <v>810</v>
+      </c>
+      <c r="F5" s="3">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3">
+        <v>570</v>
+      </c>
+      <c r="K5" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3">
+        <v>570</v>
+      </c>
+      <c r="C6" s="3">
+        <v>810</v>
+      </c>
+      <c r="D6" s="2">
+        <v>570</v>
+      </c>
+      <c r="E6" s="2">
+        <v>810</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3">
+        <v>570</v>
+      </c>
+      <c r="K6" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3">
+        <v>570</v>
+      </c>
+      <c r="C7" s="3">
+        <v>810</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>570</v>
+      </c>
+      <c r="I7" s="3">
+        <v>810</v>
+      </c>
+      <c r="J7" s="2">
+        <v>570</v>
+      </c>
+      <c r="K7" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>570</v>
+      </c>
+      <c r="C8" s="2">
+        <v>810</v>
+      </c>
+      <c r="D8" s="3">
+        <v>570</v>
+      </c>
+      <c r="E8" s="3">
+        <v>810</v>
+      </c>
+      <c r="F8" s="3">
+        <v>570</v>
+      </c>
+      <c r="G8" s="3">
+        <v>810</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3">
+        <v>0</v>
+      </c>
+      <c r="K8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3">
+        <v>570</v>
+      </c>
+      <c r="C9" s="3">
+        <v>810</v>
+      </c>
+      <c r="D9" s="2">
+        <v>570</v>
+      </c>
+      <c r="E9" s="2">
+        <v>810</v>
+      </c>
+      <c r="F9" s="3">
+        <v>570</v>
+      </c>
+      <c r="G9" s="3">
+        <v>810</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3">
+        <v>570</v>
+      </c>
+      <c r="C10" s="3">
+        <v>810</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
+        <v>570</v>
+      </c>
+      <c r="I10" s="2">
+        <v>810</v>
+      </c>
+      <c r="J10" s="3">
+        <v>570</v>
+      </c>
+      <c r="K10" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>570</v>
+      </c>
+      <c r="G11" s="2">
+        <v>810</v>
+      </c>
+      <c r="H11" s="3">
+        <v>570</v>
+      </c>
+      <c r="I11" s="3">
+        <v>810</v>
+      </c>
+      <c r="J11" s="3">
+        <v>570</v>
+      </c>
+      <c r="K11" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3">
+        <v>570</v>
+      </c>
+      <c r="C12" s="3">
+        <v>810</v>
+      </c>
+      <c r="D12" s="2">
+        <v>570</v>
+      </c>
+      <c r="E12" s="2">
+        <v>810</v>
+      </c>
+      <c r="F12" s="3">
+        <v>570</v>
+      </c>
+      <c r="G12" s="3">
+        <v>810</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0</v>
+      </c>
+      <c r="J12" s="3">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>570</v>
+      </c>
+      <c r="C13" s="2">
+        <v>810</v>
+      </c>
+      <c r="D13" s="3">
+        <v>570</v>
+      </c>
+      <c r="E13" s="3">
+        <v>810</v>
+      </c>
+      <c r="F13" s="3">
+        <v>570</v>
+      </c>
+      <c r="G13" s="3">
+        <v>810</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3">
+        <v>0</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>570</v>
+      </c>
+      <c r="E14" s="3">
+        <v>810</v>
+      </c>
+      <c r="F14" s="2">
+        <v>570</v>
+      </c>
+      <c r="G14" s="2">
+        <v>810</v>
+      </c>
+      <c r="H14" s="3">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3">
+        <v>570</v>
+      </c>
+      <c r="K14" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0</v>
+      </c>
+      <c r="D15" s="3">
+        <v>570</v>
+      </c>
+      <c r="E15" s="3">
+        <v>810</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0</v>
+      </c>
+      <c r="H15" s="3">
+        <v>570</v>
+      </c>
+      <c r="I15" s="3">
+        <v>810</v>
+      </c>
+      <c r="J15" s="2">
+        <v>570</v>
+      </c>
+      <c r="K15" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3">
+        <v>570</v>
+      </c>
+      <c r="E16" s="3">
+        <v>810</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>570</v>
+      </c>
+      <c r="I16" s="2">
+        <v>810</v>
+      </c>
+      <c r="J16" s="3">
+        <v>570</v>
+      </c>
+      <c r="K16" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3">
+        <v>570</v>
+      </c>
+      <c r="C17" s="3">
+        <v>810</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3">
+        <v>570</v>
+      </c>
+      <c r="G17" s="3">
+        <v>810</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>570</v>
+      </c>
+      <c r="K17" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2">
+        <v>570</v>
+      </c>
+      <c r="C18" s="2">
+        <v>810</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3">
+        <v>570</v>
+      </c>
+      <c r="G18" s="3">
+        <v>810</v>
+      </c>
+      <c r="H18" s="3">
+        <v>570</v>
+      </c>
+      <c r="I18" s="3">
+        <v>810</v>
+      </c>
+      <c r="J18" s="3">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3">
+        <v>0</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2">
+        <v>570</v>
+      </c>
+      <c r="E19" s="2">
+        <v>810</v>
+      </c>
+      <c r="F19" s="3">
+        <v>570</v>
+      </c>
+      <c r="G19" s="3">
+        <v>810</v>
+      </c>
+      <c r="H19" s="3">
+        <v>0</v>
+      </c>
+      <c r="I19" s="3">
+        <v>0</v>
+      </c>
+      <c r="J19" s="3">
+        <v>570</v>
+      </c>
+      <c r="K19" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3">
+        <v>570</v>
+      </c>
+      <c r="C20" s="3">
+        <v>810</v>
+      </c>
+      <c r="D20" s="3">
+        <v>570</v>
+      </c>
+      <c r="E20" s="3">
+        <v>810</v>
+      </c>
+      <c r="F20" s="2">
+        <v>570</v>
+      </c>
+      <c r="G20" s="2">
+        <v>810</v>
+      </c>
+      <c r="H20" s="3">
+        <v>0</v>
+      </c>
+      <c r="I20" s="3">
+        <v>0</v>
+      </c>
+      <c r="J20" s="3">
+        <v>0</v>
+      </c>
+      <c r="K20" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3">
+        <v>570</v>
+      </c>
+      <c r="C21" s="3">
+        <v>810</v>
+      </c>
+      <c r="D21" s="3">
+        <v>570</v>
+      </c>
+      <c r="E21" s="3">
+        <v>810</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
+        <v>570</v>
+      </c>
+      <c r="I21" s="2">
+        <v>810</v>
+      </c>
+      <c r="J21" s="3">
+        <v>0</v>
+      </c>
+      <c r="K21" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3">
+        <v>570</v>
+      </c>
+      <c r="C22" s="3">
+        <v>810</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2">
+        <v>570</v>
+      </c>
+      <c r="G22" s="2">
+        <v>810</v>
+      </c>
+      <c r="H22" s="3">
+        <v>570</v>
+      </c>
+      <c r="I22" s="3">
+        <v>810</v>
+      </c>
+      <c r="J22" s="3">
+        <v>0</v>
+      </c>
+      <c r="K22" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3">
+        <v>570</v>
+      </c>
+      <c r="E23" s="3">
+        <v>810</v>
+      </c>
+      <c r="F23" s="3">
+        <v>570</v>
+      </c>
+      <c r="G23" s="3">
+        <v>810</v>
+      </c>
+      <c r="H23" s="2">
+        <v>570</v>
+      </c>
+      <c r="I23" s="2">
+        <v>810</v>
+      </c>
+      <c r="J23" s="3">
+        <v>0</v>
+      </c>
+      <c r="K23" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2">
+        <v>570</v>
+      </c>
+      <c r="C24" s="2">
+        <v>810</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3">
+        <v>570</v>
+      </c>
+      <c r="G24" s="3">
+        <v>810</v>
+      </c>
+      <c r="H24" s="3">
+        <v>0</v>
+      </c>
+      <c r="I24" s="3">
+        <v>0</v>
+      </c>
+      <c r="J24" s="3">
+        <v>570</v>
+      </c>
+      <c r="K24" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3">
+        <v>0</v>
+      </c>
+      <c r="C25" s="3">
+        <v>0</v>
+      </c>
+      <c r="D25" s="3">
+        <v>570</v>
+      </c>
+      <c r="E25" s="3">
+        <v>810</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0</v>
+      </c>
+      <c r="H25" s="3">
+        <v>570</v>
+      </c>
+      <c r="I25" s="3">
+        <v>810</v>
+      </c>
+      <c r="J25" s="2">
+        <v>570</v>
+      </c>
+      <c r="K25" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3">
+        <v>0</v>
+      </c>
+      <c r="C26" s="3">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2">
+        <v>570</v>
+      </c>
+      <c r="E26" s="2">
+        <v>810</v>
+      </c>
+      <c r="F26" s="3">
+        <v>570</v>
+      </c>
+      <c r="G26" s="3">
+        <v>810</v>
+      </c>
+      <c r="H26" s="3">
+        <v>0</v>
+      </c>
+      <c r="I26" s="3">
+        <v>0</v>
+      </c>
+      <c r="J26" s="3">
+        <v>570</v>
+      </c>
+      <c r="K26" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3">
+        <v>570</v>
+      </c>
+      <c r="C27" s="3">
+        <v>810</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3">
+        <v>0</v>
+      </c>
+      <c r="F27" s="3">
+        <v>570</v>
+      </c>
+      <c r="G27" s="3">
+        <v>810</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2">
+        <v>570</v>
+      </c>
+      <c r="K27" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2">
+        <v>570</v>
+      </c>
+      <c r="C28" s="2">
+        <v>810</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3">
+        <v>0</v>
+      </c>
+      <c r="F28" s="3">
+        <v>0</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
+      <c r="H28" s="3">
+        <v>570</v>
+      </c>
+      <c r="I28" s="3">
+        <v>810</v>
+      </c>
+      <c r="J28" s="3">
+        <v>570</v>
+      </c>
+      <c r="K28" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0</v>
+      </c>
+      <c r="D29" s="2">
+        <v>570</v>
+      </c>
+      <c r="E29" s="2">
+        <v>810</v>
+      </c>
+      <c r="F29" s="3">
+        <v>0</v>
+      </c>
+      <c r="G29" s="3">
+        <v>0</v>
+      </c>
+      <c r="H29" s="3">
+        <v>570</v>
+      </c>
+      <c r="I29" s="3">
+        <v>810</v>
+      </c>
+      <c r="J29" s="3">
+        <v>570</v>
+      </c>
+      <c r="K29" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3">
+        <v>570</v>
+      </c>
+      <c r="C30" s="3">
+        <v>810</v>
+      </c>
+      <c r="D30" s="3">
+        <v>570</v>
+      </c>
+      <c r="E30" s="3">
+        <v>810</v>
+      </c>
+      <c r="F30" s="2">
+        <v>570</v>
+      </c>
+      <c r="G30" s="2">
+        <v>810</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0</v>
+      </c>
+      <c r="I30" s="3">
+        <v>0</v>
+      </c>
+      <c r="J30" s="3">
+        <v>0</v>
+      </c>
+      <c r="K30" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3">
+        <v>570</v>
+      </c>
+      <c r="C31" s="3">
+        <v>810</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3">
+        <v>0</v>
+      </c>
+      <c r="F31" s="3">
+        <v>570</v>
+      </c>
+      <c r="G31" s="3">
+        <v>810</v>
+      </c>
+      <c r="H31" s="2">
+        <v>570</v>
+      </c>
+      <c r="I31" s="2">
+        <v>810</v>
+      </c>
+      <c r="J31" s="3">
+        <v>0</v>
+      </c>
+      <c r="K31" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3">
+        <v>570</v>
+      </c>
+      <c r="C32" s="3">
+        <v>810</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2">
+        <v>570</v>
+      </c>
+      <c r="G32" s="2">
+        <v>810</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0</v>
+      </c>
+      <c r="I32" s="3">
+        <v>0</v>
+      </c>
+      <c r="J32" s="3">
+        <v>570</v>
+      </c>
+      <c r="K32" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3">
+        <v>570</v>
+      </c>
+      <c r="C33" s="3">
+        <v>810</v>
+      </c>
+      <c r="D33" s="3">
+        <v>570</v>
+      </c>
+      <c r="E33" s="3">
+        <v>810</v>
+      </c>
+      <c r="F33" s="3">
+        <v>0</v>
+      </c>
+      <c r="G33" s="3">
+        <v>0</v>
+      </c>
+      <c r="H33" s="2">
+        <v>570</v>
+      </c>
+      <c r="I33" s="2">
+        <v>810</v>
+      </c>
+      <c r="J33" s="3">
+        <v>0</v>
+      </c>
+      <c r="K33" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3">
+        <v>0</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0</v>
+      </c>
+      <c r="E34" s="3">
+        <v>0</v>
+      </c>
+      <c r="F34" s="3">
+        <v>570</v>
+      </c>
+      <c r="G34" s="3">
+        <v>810</v>
+      </c>
+      <c r="H34" s="3">
+        <v>570</v>
+      </c>
+      <c r="I34" s="3">
+        <v>810</v>
+      </c>
+      <c r="J34" s="2">
+        <v>570</v>
+      </c>
+      <c r="K34" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2">
+        <v>570</v>
+      </c>
+      <c r="C35" s="2">
+        <v>810</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3">
+        <v>0</v>
+      </c>
+      <c r="F35" s="3">
+        <v>0</v>
+      </c>
+      <c r="G35" s="3">
+        <v>0</v>
+      </c>
+      <c r="H35" s="3">
+        <v>570</v>
+      </c>
+      <c r="I35" s="3">
+        <v>810</v>
+      </c>
+      <c r="J35" s="3">
+        <v>570</v>
+      </c>
+      <c r="K35" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3">
+        <v>0</v>
+      </c>
+      <c r="D36" s="2">
+        <v>570</v>
+      </c>
+      <c r="E36" s="2">
+        <v>810</v>
+      </c>
+      <c r="F36" s="3">
+        <v>570</v>
+      </c>
+      <c r="G36" s="3">
+        <v>810</v>
+      </c>
+      <c r="H36" s="3">
+        <v>570</v>
+      </c>
+      <c r="I36" s="3">
+        <v>810</v>
+      </c>
+      <c r="J36" s="3">
+        <v>0</v>
+      </c>
+      <c r="K36" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3">
+        <v>570</v>
+      </c>
+      <c r="C37" s="3">
+        <v>810</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3">
+        <v>0</v>
+      </c>
+      <c r="F37" s="3">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3">
+        <v>0</v>
+      </c>
+      <c r="H37" s="3">
+        <v>570</v>
+      </c>
+      <c r="I37" s="3">
+        <v>810</v>
+      </c>
+      <c r="J37" s="2">
+        <v>570</v>
+      </c>
+      <c r="K37" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2">
+        <v>570</v>
+      </c>
+      <c r="C38" s="2">
+        <v>810</v>
+      </c>
+      <c r="D38" s="3">
+        <v>570</v>
+      </c>
+      <c r="E38" s="3">
+        <v>810</v>
+      </c>
+      <c r="F38" s="3">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3">
+        <v>0</v>
+      </c>
+      <c r="H38" s="3">
+        <v>570</v>
+      </c>
+      <c r="I38" s="3">
+        <v>810</v>
+      </c>
+      <c r="J38" s="3">
+        <v>0</v>
+      </c>
+      <c r="K38" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3">
+        <v>0</v>
+      </c>
+      <c r="D39" s="2">
+        <v>570</v>
+      </c>
+      <c r="E39" s="2">
+        <v>810</v>
+      </c>
+      <c r="F39" s="3">
+        <v>570</v>
+      </c>
+      <c r="G39" s="3">
+        <v>810</v>
+      </c>
+      <c r="H39" s="3">
+        <v>570</v>
+      </c>
+      <c r="I39" s="3">
+        <v>810</v>
+      </c>
+      <c r="J39" s="3">
+        <v>0</v>
+      </c>
+      <c r="K39" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3">
+        <v>0</v>
+      </c>
+      <c r="C40" s="3">
+        <v>0</v>
+      </c>
+      <c r="D40" s="3">
+        <v>570</v>
+      </c>
+      <c r="E40" s="3">
+        <v>810</v>
+      </c>
+      <c r="F40" s="2">
+        <v>570</v>
+      </c>
+      <c r="G40" s="2">
+        <v>810</v>
+      </c>
+      <c r="H40" s="3">
+        <v>570</v>
+      </c>
+      <c r="I40" s="3">
+        <v>810</v>
+      </c>
+      <c r="J40" s="3">
+        <v>0</v>
+      </c>
+      <c r="K40" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3">
+        <v>0</v>
+      </c>
+      <c r="C41" s="3">
+        <v>0</v>
+      </c>
+      <c r="D41" s="3">
+        <v>0</v>
+      </c>
+      <c r="E41" s="3">
+        <v>0</v>
+      </c>
+      <c r="F41" s="3">
+        <v>570</v>
+      </c>
+      <c r="G41" s="3">
+        <v>810</v>
+      </c>
+      <c r="H41" s="2">
+        <v>570</v>
+      </c>
+      <c r="I41" s="2">
+        <v>810</v>
+      </c>
+      <c r="J41" s="3">
+        <v>570</v>
+      </c>
+      <c r="K41" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3">
+        <v>570</v>
+      </c>
+      <c r="C42" s="3">
+        <v>810</v>
+      </c>
+      <c r="D42" s="2">
+        <v>570</v>
+      </c>
+      <c r="E42" s="2">
+        <v>810</v>
+      </c>
+      <c r="F42" s="3">
+        <v>0</v>
+      </c>
+      <c r="G42" s="3">
+        <v>0</v>
+      </c>
+      <c r="H42" s="3">
+        <v>0</v>
+      </c>
+      <c r="I42" s="3">
+        <v>0</v>
+      </c>
+      <c r="J42" s="3">
+        <v>570</v>
+      </c>
+      <c r="K42" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3">
+        <v>0</v>
+      </c>
+      <c r="C43" s="3">
+        <v>0</v>
+      </c>
+      <c r="D43" s="3">
+        <v>570</v>
+      </c>
+      <c r="E43" s="3">
+        <v>810</v>
+      </c>
+      <c r="F43" s="2">
+        <v>570</v>
+      </c>
+      <c r="G43" s="2">
+        <v>810</v>
+      </c>
+      <c r="H43" s="3">
+        <v>570</v>
+      </c>
+      <c r="I43" s="3">
+        <v>810</v>
+      </c>
+      <c r="J43" s="3">
+        <v>0</v>
+      </c>
+      <c r="K43" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3">
+        <v>570</v>
+      </c>
+      <c r="C44" s="3">
+        <v>810</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0</v>
+      </c>
+      <c r="E44" s="3">
+        <v>0</v>
+      </c>
+      <c r="F44" s="3">
+        <v>570</v>
+      </c>
+      <c r="G44" s="3">
+        <v>810</v>
+      </c>
+      <c r="H44" s="2">
+        <v>570</v>
+      </c>
+      <c r="I44" s="2">
+        <v>810</v>
+      </c>
+      <c r="J44" s="3">
+        <v>0</v>
+      </c>
+      <c r="K44" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3">
+        <v>0</v>
+      </c>
+      <c r="C45" s="3">
+        <v>0</v>
+      </c>
+      <c r="D45" s="3">
+        <v>570</v>
+      </c>
+      <c r="E45" s="3">
+        <v>810</v>
+      </c>
+      <c r="F45" s="3">
+        <v>0</v>
+      </c>
+      <c r="G45" s="3">
+        <v>0</v>
+      </c>
+      <c r="H45" s="3">
+        <v>570</v>
+      </c>
+      <c r="I45" s="3">
+        <v>810</v>
+      </c>
+      <c r="J45" s="2">
+        <v>570</v>
+      </c>
+      <c r="K45" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2">
+        <v>570</v>
+      </c>
+      <c r="C46" s="2">
+        <v>810</v>
+      </c>
+      <c r="D46" s="3">
+        <v>0</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0</v>
+      </c>
+      <c r="F46" s="3">
+        <v>0</v>
+      </c>
+      <c r="G46" s="3">
+        <v>0</v>
+      </c>
+      <c r="H46" s="3">
+        <v>570</v>
+      </c>
+      <c r="I46" s="3">
+        <v>810</v>
+      </c>
+      <c r="J46" s="3">
+        <v>570</v>
+      </c>
+      <c r="K46" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3">
+        <v>570</v>
+      </c>
+      <c r="C47" s="3">
+        <v>810</v>
+      </c>
+      <c r="D47" s="2">
+        <v>570</v>
+      </c>
+      <c r="E47" s="2">
+        <v>810</v>
+      </c>
+      <c r="F47" s="3">
+        <v>570</v>
+      </c>
+      <c r="G47" s="3">
+        <v>810</v>
+      </c>
+      <c r="H47" s="3">
+        <v>0</v>
+      </c>
+      <c r="I47" s="3">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3">
+        <v>0</v>
+      </c>
+      <c r="K47" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3">
+        <v>0</v>
+      </c>
+      <c r="C48" s="3">
+        <v>0</v>
+      </c>
+      <c r="D48" s="3">
+        <v>0</v>
+      </c>
+      <c r="E48" s="3">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2">
+        <v>570</v>
+      </c>
+      <c r="G48" s="2">
+        <v>810</v>
+      </c>
+      <c r="H48" s="3">
+        <v>570</v>
+      </c>
+      <c r="I48" s="3">
+        <v>810</v>
+      </c>
+      <c r="J48" s="3">
+        <v>570</v>
+      </c>
+      <c r="K48" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3">
+        <v>0</v>
+      </c>
+      <c r="C49" s="3">
+        <v>0</v>
+      </c>
+      <c r="D49" s="3">
+        <v>570</v>
+      </c>
+      <c r="E49" s="3">
+        <v>810</v>
+      </c>
+      <c r="F49" s="3">
+        <v>0</v>
+      </c>
+      <c r="G49" s="3">
+        <v>0</v>
+      </c>
+      <c r="H49" s="2">
+        <v>570</v>
+      </c>
+      <c r="I49" s="2">
+        <v>810</v>
+      </c>
+      <c r="J49" s="3">
+        <v>570</v>
+      </c>
+      <c r="K49" s="3">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3">
+        <v>570</v>
+      </c>
+      <c r="C50" s="3">
+        <v>810</v>
+      </c>
+      <c r="D50" s="3">
+        <v>570</v>
+      </c>
+      <c r="E50" s="3">
+        <v>810</v>
+      </c>
+      <c r="F50" s="3">
+        <v>0</v>
+      </c>
+      <c r="G50" s="3">
+        <v>0</v>
+      </c>
+      <c r="H50" s="3">
+        <v>0</v>
+      </c>
+      <c r="I50" s="3">
+        <v>0</v>
+      </c>
+      <c r="J50" s="2">
+        <v>570</v>
+      </c>
+      <c r="K50" s="2">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2">
+        <v>570</v>
+      </c>
+      <c r="C51" s="2">
+        <v>810</v>
+      </c>
+      <c r="D51" s="3">
+        <v>570</v>
+      </c>
+      <c r="E51" s="3">
+        <v>810</v>
+      </c>
+      <c r="F51" s="3">
+        <v>570</v>
+      </c>
+      <c r="G51" s="3">
+        <v>810</v>
+      </c>
+      <c r="H51" s="3">
+        <v>0</v>
+      </c>
+      <c r="I51" s="3">
+        <v>0</v>
+      </c>
+      <c r="J51" s="3">
+        <v>0</v>
+      </c>
+      <c r="K51" s="3">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>